<commit_message>
feat: add CMR package with CMR_GetCustomerByID flow service
- IS package structure: CMR/manifest.v3
- Service: CustomerService:CMR_GetCustomerByID
- Flow file: fetchCustomer.flow (named per request)
- HTTP GET to localhost:5001/customers/{customer_id}
- TRY/CATCH with IF 200 / ELSEIF 404 / ELSE routing
- UTF-8 byte decoding, JSON parse, name concat
- Documentation: CMR_GetCustomerByID.md with Mermaid diagram
- Removed deleted customerService_GetCustomerByID artefacts
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/subkumak/bob-workspace/flowpilot-demo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41455037-D724-624F-8192-D1DD0408DE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED11C2D6-B348-9840-A632-DF2903287491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="24640" xr2:uid="{88332C4F-0D0A-7D4E-8F2E-B786A235A8C3}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Create a new webMethods Flow service named customWriteToLog.
 Implement the following sequence of steps:
@@ -103,10 +103,13 @@
     <t>https://yourlearning.ibm.com/activity/ITS-ZM410G</t>
   </si>
   <si>
-    <t>Create a webMethods Flow Service named customerService_GetCustomerByID in namespace CustomerService. Define input string customer_id and outputs string name, email, accountStatus, errorMessage. Perform an HTTP GET to http://localhost:5001/customers/{customer_id} (replace {customer_id} with the input). Capture HTTP status and response body (bytes). Convert response bytes to a UTF-8 string and, if status == 200, parse the JSON, set name = first_name + ' ' + last_name, email = email, accountStatus = status, and set errorMessage = ''. If status == 404 set errorMessage = 'Customer not found' and clear other outputs. For any other status or on exception set errorMessage = 'Customer API unavailable' and clear other outputs. Wrap operations in try/catch. Implement using valid webMethods Flow Service DSL constructs, proper variable names, and correct conditional expressions.</t>
-  </si>
-  <si>
     <t>Working</t>
+  </si>
+  <si>
+    <t>Create a test suite for the customerService_GetCustomerByID with full non-regression coverage by enumerating through all the different scenarios for  the flow services.</t>
+  </si>
+  <si>
+    <t>Create a webMethods Flow Service named customerService_GetCustomerByID in namespace CustomerService. Define input string customer_id and outputs string name, email, accountStatus, errorMessage. Perform an HTTP GET to http://localhost:5001/customers/{customer_id} (replace {customer_id} with the input). Capture HTTP status and response body (bytes). Convert response bytes to a UTF-8 string and, if status == 200, parse the JSON, set name = first_name + ' ' + last_name, email = email, accountStatus = status, and set errorMessage = ''. If status == 404 set errorMessage = 'Customer not found' and clear other outputs. For any other status or on exception set errorMessage = 'Customer API unavailable' and clear other outputs. Wrap operations in try/catch. Implement using valid webMethods Flow Service DSL constructs, proper variable names, and correct conditional expressions."Name the flow file fetchCustomer.flow" and document a service.</t>
   </si>
 </sst>
 </file>
@@ -492,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FD756CC-FDC2-F941-B6EB-46E7F6FCA847}">
-  <dimension ref="B4:C25"/>
+  <dimension ref="B4:C28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="85" customWidth="1"/>
@@ -541,9 +544,14 @@
     </row>
     <row r="25" spans="2:3" ht="170" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" t="s">
         <v>19</v>
       </c>
-      <c r="C25" t="s">
+    </row>
+    <row r="28" spans="2:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B28" s="1" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: CustomerService IWHI package with fetchCustomer flow service
Package structure (mirrors CurrencyExchange reference package):
  CustomerService/
    manifest.v3         — IS package manifest (correct Values schema)
    assets.json         — package asset registry
    pub/index.html      — web descriptor
    ns/
      CustomerService/
        node.idf        — namespace registry
        fetchCustomer/
          fetchCustomer.flow  — FSL flow service

Service: CustomerService:fetchCustomer
  Input:  customer_id (String)
  Output: name, email, accountStatus, errorMessage (String)
  - HTTP GET http://localhost:5001/customers/{customer_id}
  - UTF-8 decode, JSON parse on HTTP 200
  - name = first_name + space + last_name
  - IF 200 / ELSEIF 404 / ELSE / TRY-CATCH error handling
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/subkumak/bob-workspace/flowpilot-demo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED11C2D6-B348-9840-A632-DF2903287491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB641805-EF6D-7546-9485-796653D35E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="24640" xr2:uid="{88332C4F-0D0A-7D4E-8F2E-B786A235A8C3}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Create a new webMethods Flow service named customWriteToLog.
 Implement the following sequence of steps:
@@ -109,7 +109,13 @@
     <t>Create a test suite for the customerService_GetCustomerByID with full non-regression coverage by enumerating through all the different scenarios for  the flow services.</t>
   </si>
   <si>
-    <t>Create a webMethods Flow Service named customerService_GetCustomerByID in namespace CustomerService. Define input string customer_id and outputs string name, email, accountStatus, errorMessage. Perform an HTTP GET to http://localhost:5001/customers/{customer_id} (replace {customer_id} with the input). Capture HTTP status and response body (bytes). Convert response bytes to a UTF-8 string and, if status == 200, parse the JSON, set name = first_name + ' ' + last_name, email = email, accountStatus = status, and set errorMessage = ''. If status == 404 set errorMessage = 'Customer not found' and clear other outputs. For any other status or on exception set errorMessage = 'Customer API unavailable' and clear other outputs. Wrap operations in try/catch. Implement using valid webMethods Flow Service DSL constructs, proper variable names, and correct conditional expressions."Name the flow file fetchCustomer.flow" and document a service.</t>
+    <t>Create a webMethods Flow Service named customerService_GetCustomerByID in namespace CustomerService. Define input string customer_id and outputs string name, email, accountStatus, errorMessage. Perform an HTTP GET to http://localhost:5001/customers/{customer_id} (replace {customer_id} with the input). Capture HTTP status and response body (bytes). Convert response bytes to a UTF-8 string and, if status == 200, parse the JSON, set name = first_name + ' ' + last_name, email = email, accountStatus = status, and set errorMessage = ''. If status == 404 set errorMessage = 'Customer not found' and clear other outputs. For any other status or on exception set errorMessage = 'Customer API unavailable' and clear other outputs. Wrap operations in try/catch. Implement using valid webMethods Flow Service DSL constructs, proper variable names, and correct conditional expressions."Name the flow file as  fetchCustomer.flow" and document a service. Please generate the complete package structure with all necessary files.</t>
+  </si>
+  <si>
+    <t>Create a complete webMethods Integration Server package named `CustomerService_GetCustomerByIDProject` containing a Flow Service named  `fetchCustomer.flow`, and the document the service.  Define input string customer_id and outputs string name, email, accountStatus, errorMessage. Perform an HTTP GET to http://localhost:5001/customers/{customer_id} (replace {customer_id} with the input). Capture HTTP status and response body (bytes). Convert response bytes to a UTF-8 string and, if status == 200, parse the JSON, set name = first_name + ' ' + last_name, email = email, accountStatus = status, and set errorMessage = ''. If status == 404 set errorMessage = 'Customer not found' and clear other outputs. For any other status or on exception set errorMessage = 'Customer API unavailable' and clear other outputs. Wrap operations in try/catch. Implement using valid webMethods Flow Service DSL constructs, proper variable names, and correct conditional expressions.</t>
+  </si>
+  <si>
+    <t>Create a  Flow Service named  `fetchCustomer.flow` and the document the service.   The service accepts a input string customer_id and outputs string name, email, accountStatus, errorMessage. Perform an HTTP GET to REST API endpoint  http://localhost:5001/customers/{customer_id} (replace {customer_id} with the input). Capture HTTP status and response body (bytes). Convert response bytes to a UTF-8 string and, if status == 200, parse the JSON, set name = first_name + ' ' + last_name, email = email, accountStatus = status, and set errorMessage = ''. If status == 404 set errorMessage = 'Customer not found' and clear other outputs. For any other status or on exception set errorMessage = 'Customer API unavailable' and clear other outputs. Wrap operations in try/catch. Implement using valid webMethods Flow Service DSL constructs, proper variable names, and correct conditional expressions.</t>
   </si>
 </sst>
 </file>
@@ -495,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FD756CC-FDC2-F941-B6EB-46E7F6FCA847}">
-  <dimension ref="B4:C28"/>
+  <dimension ref="B4:C34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="85" customWidth="1"/>
@@ -542,7 +548,7 @@
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" s="1"/>
     </row>
-    <row r="25" spans="2:3" ht="170" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:3" ht="187" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
         <v>21</v>
       </c>
@@ -553,6 +559,16 @@
     <row r="28" spans="2:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B28" s="1" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" ht="187" x14ac:dyDescent="0.2">
+      <c r="B30" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" ht="170" x14ac:dyDescent="0.2">
+      <c r="B34" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>